<commit_message>
Polish single-sheet buyer database layout
Title banner, KPI summary cards, color legend, centered short columns,
row heights sized to content, one phone/email per line, short link text,
and A4 landscape print setup.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0119C5FjC7uP8a9Ri21UaXKa
</commit_message>
<xml_diff>
--- a/Database_Buyer_Manggis_1Sheet.xlsx
+++ b/Database_Buyer_Manggis_1Sheet.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Buyer Manggis" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Buyer Manggis'!$4:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Buyer Manggis'!$10:$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd-mmm-yy"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,8 +32,34 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
       <color rgb="001F3864"/>
-      <sz val="14"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -53,12 +79,17 @@
     </font>
     <font>
       <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <color rgb="000563C1"/>
       <sz val="10"/>
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -67,11 +98,46 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002F5597"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF1FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDEDED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8CBAD"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -79,40 +145,89 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <top style="medium">
+        <color rgb="002F5597"/>
+      </top>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="6">
     <dxf>
       <font>
         <name val="Arial"/>
@@ -142,7 +257,7 @@
       </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00F2F2F2"/>
+          <fgColor rgb="00EDEDED"/>
         </patternFill>
       </fill>
     </dxf>
@@ -157,13 +272,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00F2F2F2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -247,9 +355,34 @@
 </styleSheet>
 </file>
 
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Catatan</author>
+  </authors>
+  <commentList>
+    <comment ref="M39" authorId="0" shapeId="0">
+      <text>
+        <t>Tinggi (alamat), Sedang (email)</t>
+      </text>
+    </comment>
+    <comment ref="M48" authorId="0" shapeId="0">
+      <text>
+        <t>Tinggi (telp/alamat), Sedang (email)</t>
+      </text>
+    </comment>
+    <comment ref="M54" authorId="0" shapeId="0">
+      <text>
+        <t>Tinggi (email), Sedang (telp/alamat)</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblBuyerManggis" displayName="tblBuyerManggis" ref="A4:P49" headerRowCount="1">
-  <autoFilter ref="A4:P49"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblBuyerManggis" displayName="tblBuyerManggis" ref="A10:P55" headerRowCount="1">
+  <autoFilter ref="A10:P55"/>
   <tableColumns count="16">
     <tableColumn id="1" name="No"/>
     <tableColumn id="2" name="Perusahaan"/>
@@ -262,13 +395,13 @@
     <tableColumn id="9" name="Email"/>
     <tableColumn id="10" name="Telepon"/>
     <tableColumn id="11" name="Alamat"/>
-    <tableColumn id="12" name="Halaman Kontak / Sumber"/>
-    <tableColumn id="13" name="Keyakinan Kontak"/>
+    <tableColumn id="12" name="Link Kontak"/>
+    <tableColumn id="13" name="Keyakinan"/>
     <tableColumn id="14" name="Status"/>
     <tableColumn id="15" name="Follow-up"/>
     <tableColumn id="16" name="Catatan"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="0"/>
 </table>
 </file>
 
@@ -558,3004 +691,3177 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F3864"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P49"/>
+  <dimension ref="A1:P55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="26" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
-    <col width="34" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="38" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>DATABASE BUYER MANGGIS SEGAR: CHINA, HONG KONG &amp; TIMUR TENGAH</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+          <t xml:space="preserve">  DATABASE BUYER MANGGIS SEGAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prioritas A = terbukti impor manggis · B = importir buah tropis · C = prospek sekunder   |   Keyakinan: Tinggi = situs resmi · Sedang = direktori pihak ketiga   |   Kolom kuning = diisi Anda   |   Riset 27 Sep 2026: cek ulang kontak sebelum kirim penawaran</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+          <t xml:space="preserve">  China · Hong Kong · UAE · Saudi Arabia · Qatar · Kuwait · Oman · Bahrain   |   Riset sumber publik, 27 Sep 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="10" customHeight="1"/>
+    <row r="4" ht="18" customHeight="1">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Total Buyer</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>China &amp; Hong Kong</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Timur Tengah</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Prioritas A</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="n"/>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Punya Email</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="n"/>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>Sudah Dihubungi</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="n"/>
+      <c r="N4" s="4" t="n"/>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>Deal</t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="B5" s="5">
+        <f>COUNTA($B$11:$B$255)</f>
+        <v/>
+      </c>
+      <c r="C5" s="5">
+        <f>COUNTIF($C$11:$C$255,"China")+COUNTIF($C$11:$C$255,"Hong Kong")</f>
+        <v/>
+      </c>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="5">
+        <f>COUNTA($B$11:$B$255)-COUNTIF($C$11:$C$255,"China")-COUNTIF($C$11:$C$255,"Hong Kong")</f>
+        <v/>
+      </c>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="5">
+        <f>COUNTIF($F$11:$F$255,"A")</f>
+        <v/>
+      </c>
+      <c r="I5" s="6" t="n"/>
+      <c r="J5" s="5">
+        <f>COUNTIF($I$11:$I$255,"?*")</f>
+        <v/>
+      </c>
+      <c r="K5" s="6" t="n"/>
+      <c r="L5" s="5">
+        <f>COUNTA($B$11:$B$255)-COUNTIF($N$11:$N$255,"Baru")</f>
+        <v/>
+      </c>
+      <c r="M5" s="6" t="n"/>
+      <c r="N5" s="6" t="n"/>
+      <c r="O5" s="5">
+        <f>COUNTIF($N$11:$N$255,"Deal")</f>
+        <v/>
+      </c>
+      <c r="P5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="10" customHeight="1"/>
+    <row r="7" ht="20" customHeight="1">
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>A  ·  Terbukti impor manggis</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="9" t="n"/>
+      <c r="F7" s="10" t="inlineStr">
+        <is>
+          <t>B  ·  Importir buah tropis</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="n"/>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>C  ·  Prospek sekunder</t>
+        </is>
+      </c>
+      <c r="I7" s="13" t="n"/>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>Kolom kuning = diisi Anda</t>
+        </is>
+      </c>
+      <c r="K7" s="15" t="n"/>
+      <c r="L7" s="16" t="inlineStr">
+        <is>
+          <t>Follow-up jatuh tempo</t>
+        </is>
+      </c>
+      <c r="M7" s="17" t="n"/>
+      <c r="N7" s="17" t="n"/>
+      <c r="O7" s="8" t="inlineStr">
+        <is>
+          <t>Status Deal</t>
+        </is>
+      </c>
+      <c r="P7" s="9" t="n"/>
+    </row>
+    <row r="8">
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Keyakinan kontak: Tinggi = dari situs resmi perusahaan · Sedang = dari direktori/data dagang pihak ketiga. Konfirmasi kontak sebelum mengirim penawaran harga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="8" customHeight="1"/>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>Perusahaan</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C10" s="19" t="inlineStr">
         <is>
           <t>Negara</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D10" s="19" t="inlineStr">
         <is>
           <t>Kota</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E10" s="19" t="inlineStr">
         <is>
           <t>Tipe</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F10" s="19" t="inlineStr">
         <is>
           <t>Prioritas</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G10" s="19" t="inlineStr">
         <is>
           <t>Produk / Fokus</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H10" s="19" t="inlineStr">
         <is>
           <t>PIC</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="I10" s="19" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="J10" s="19" t="inlineStr">
         <is>
           <t>Telepon</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K10" s="19" t="inlineStr">
         <is>
           <t>Alamat</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>Halaman Kontak / Sumber</t>
-        </is>
-      </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>Keyakinan Kontak</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="L10" s="19" t="inlineStr">
+        <is>
+          <t>Link Kontak</t>
+        </is>
+      </c>
+      <c r="M10" s="19" t="inlineStr">
+        <is>
+          <t>Keyakinan</t>
+        </is>
+      </c>
+      <c r="N10" s="19" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="O10" s="19" t="inlineStr">
         <is>
           <t>Follow-up</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="P10" s="19" t="inlineStr">
         <is>
           <t>Catatan</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="4" t="n">
+    <row r="11" ht="47" customHeight="1">
+      <c r="A11" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
         <is>
           <t>Beijing Junhui International Trading Co., Ltd.</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>China</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D11" s="22" t="inlineStr">
         <is>
           <t>Beijing</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E11" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F11" s="20" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G5" s="5" t="inlineStr">
+      <c r="G11" s="22" t="inlineStr">
         <is>
           <t>Manggis dari Indonesia</t>
         </is>
       </c>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="7" t="n"/>
-      <c r="J5" s="7" t="n"/>
-      <c r="K5" s="5" t="inlineStr">
+      <c r="H11" s="23" t="n"/>
+      <c r="I11" s="23" t="n"/>
+      <c r="J11" s="23" t="n"/>
+      <c r="K11" s="22" t="inlineStr">
         <is>
           <t>No. 22121, No. 2 Baolian Street, Beijing Tianzhu Free Trade Zone, Shunyi, Beijing</t>
         </is>
       </c>
-      <c r="L5" s="8" t="inlineStr">
-        <is>
-          <t>https://en.nbd.ltd/news/d/668bd591679ff7d42846ca3410eb591e</t>
-        </is>
-      </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="L11" s="24" t="inlineStr">
+        <is>
+          <t>en.nbd.ltd</t>
+        </is>
+      </c>
+      <c r="M11" s="20" t="inlineStr">
         <is>
           <t>Sedang</t>
         </is>
       </c>
-      <c r="N5" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O5" s="9" t="n"/>
-      <c r="P5" s="6" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="n">
+      <c r="N11" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O11" s="26" t="n"/>
+      <c r="P11" s="23" t="n"/>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>Beijing Junyao International</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C12" s="20" t="inlineStr">
         <is>
           <t>China</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>Beijing</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E12" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F12" s="20" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="G12" s="22" t="inlineStr">
         <is>
           <t>Manggis segar (Indonesia, Thailand)</t>
         </is>
       </c>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="7" t="n"/>
-      <c r="J6" s="7" t="n"/>
-      <c r="K6" s="5" t="inlineStr">
+      <c r="H12" s="23" t="n"/>
+      <c r="I12" s="23" t="n"/>
+      <c r="J12" s="23" t="n"/>
+      <c r="K12" s="22" t="inlineStr">
         <is>
           <t>Room 301, Unit 4, Building N1, Nanfaxin Town, Shunyi District, Beijing 101300</t>
         </is>
       </c>
-      <c r="L6" s="8" t="inlineStr">
-        <is>
-          <t>https://www.volza.com/p/mangosteen-fruit/buyers/buyers-in-china/</t>
-        </is>
-      </c>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="L12" s="24" t="inlineStr">
+        <is>
+          <t>volza.com</t>
+        </is>
+      </c>
+      <c r="M12" s="20" t="inlineStr">
         <is>
           <t>Sedang</t>
         </is>
       </c>
-      <c r="N6" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O6" s="9" t="n"/>
-      <c r="P6" s="6" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="n">
+      <c r="N12" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O12" s="26" t="n"/>
+      <c r="P12" s="23" t="n"/>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B13" s="21" t="inlineStr">
         <is>
           <t>Chuannongjing (Hainan) International Trade Co., Ltd.</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C13" s="20" t="inlineStr">
         <is>
           <t>China</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D13" s="22" t="inlineStr">
         <is>
           <t>Hainan</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E13" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F13" s="20" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G13" s="22" t="inlineStr">
         <is>
           <t>Produk segar global, manggis</t>
         </is>
       </c>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="7" t="n"/>
-      <c r="J7" s="7" t="n"/>
-      <c r="K7" s="5" t="n"/>
-      <c r="L7" s="8" t="inlineStr">
-        <is>
-          <t>https://www.sclanghao.com/en/zhanluebuju/chuannongjing-hainan-guojimaoyiyouxiangongsi/</t>
-        </is>
-      </c>
-      <c r="M7" s="4" t="inlineStr">
-        <is>
-          <t>Tidak ditemukan</t>
-        </is>
-      </c>
-      <c r="N7" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O7" s="9" t="n"/>
-      <c r="P7" s="6" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="n">
+      <c r="H13" s="23" t="n"/>
+      <c r="I13" s="23" t="n"/>
+      <c r="J13" s="23" t="n"/>
+      <c r="K13" s="22" t="n"/>
+      <c r="L13" s="24" t="inlineStr">
+        <is>
+          <t>sclanghao.com</t>
+        </is>
+      </c>
+      <c r="M13" s="20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N13" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O13" s="26" t="n"/>
+      <c r="P13" s="23" t="n"/>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
         <is>
           <t>Goodfarmer (Jianong Food Holding Group)</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C14" s="20" t="inlineStr">
         <is>
           <t>China</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D14" s="22" t="inlineStr">
         <is>
           <t>Shanghai</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E14" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F14" s="20" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G14" s="22" t="inlineStr">
         <is>
           <t>Durian, lengkeng, manggis, pisang, nanas</t>
         </is>
       </c>
-      <c r="H8" s="6" t="n"/>
-      <c r="I8" s="7" t="n"/>
-      <c r="J8" s="7" t="n"/>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="H14" s="23" t="n"/>
+      <c r="I14" s="23" t="n"/>
+      <c r="J14" s="23" t="n"/>
+      <c r="K14" s="22" t="inlineStr">
         <is>
           <t>Area E, 11/F, No.6, Lane 2449, Jinhai Road, Pudong, Shanghai 201209</t>
         </is>
       </c>
-      <c r="L8" s="8" t="inlineStr">
-        <is>
-          <t>https://www.goodfarmer.com/en/about.html</t>
-        </is>
-      </c>
-      <c r="M8" s="4" t="inlineStr">
+      <c r="L14" s="24" t="inlineStr">
+        <is>
+          <t>goodfarmer.com</t>
+        </is>
+      </c>
+      <c r="M14" s="20" t="inlineStr">
         <is>
           <t>Sedang</t>
         </is>
       </c>
-      <c r="N8" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O8" s="9" t="n"/>
-      <c r="P8" s="6" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="n">
+      <c r="N14" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O14" s="26" t="n"/>
+      <c r="P14" s="23" t="n"/>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B15" s="21" t="inlineStr">
         <is>
           <t>Guangzhou Wen Wu He Tai Trading Co., Ltd.</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C15" s="20" t="inlineStr">
         <is>
           <t>China</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D15" s="22" t="inlineStr">
         <is>
           <t>Guangzhou</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E15" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F15" s="20" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G15" s="22" t="inlineStr">
         <is>
           <t>Buah Asia Tenggara termasuk manggis</t>
         </is>
       </c>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="n"/>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="H15" s="23" t="n"/>
+      <c r="I15" s="23" t="n"/>
+      <c r="J15" s="23" t="n"/>
+      <c r="K15" s="22" t="inlineStr">
         <is>
           <t>Shop 107, Bldg 2, No. 844 Zengcha Road, Baiyun District, Guangzhou</t>
         </is>
       </c>
-      <c r="L9" s="8" t="inlineStr">
-        <is>
-          <t>http://en.gxmfruit.com/About.aspx?ClassID=45</t>
-        </is>
-      </c>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="L15" s="24" t="inlineStr">
+        <is>
+          <t>en.gxmfruit.com</t>
+        </is>
+      </c>
+      <c r="M15" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N9" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O9" s="9" t="n"/>
-      <c r="P9" s="6" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="n">
+      <c r="N15" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O15" s="26" t="n"/>
+      <c r="P15" s="23" t="n"/>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
         <is>
           <t>Guangzhou Zhanhui Trade Co., Ltd.</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C16" s="20" t="inlineStr">
         <is>
           <t>China</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D16" s="22" t="inlineStr">
         <is>
           <t>Guangzhou</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E16" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F16" s="20" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G16" s="22" t="inlineStr">
         <is>
           <t>Durian, lengkeng, manggis Thailand; buah naga Vietnam</t>
         </is>
       </c>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="7" t="n"/>
-      <c r="J10" s="7" t="inlineStr">
+      <c r="H16" s="23" t="n"/>
+      <c r="I16" s="23" t="n"/>
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>+86 20 3433 3222</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr">
+      <c r="K16" s="22" t="inlineStr">
         <is>
           <t>No. 22, Business Tower C, Jiangnan Fruit Market, Zengcha Road, Guangzhou</t>
         </is>
       </c>
-      <c r="L10" s="8" t="inlineStr">
-        <is>
-          <t>https://www.globalsources.com/guangzhou-zhanhui/contact-us_6008834714043.htm</t>
-        </is>
-      </c>
-      <c r="M10" s="4" t="inlineStr">
+      <c r="L16" s="24" t="inlineStr">
+        <is>
+          <t>globalsources.com</t>
+        </is>
+      </c>
+      <c r="M16" s="20" t="inlineStr">
         <is>
           <t>Sedang</t>
         </is>
       </c>
-      <c r="N10" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O10" s="9" t="n"/>
-      <c r="P10" s="6" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="n">
+      <c r="N16" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O16" s="26" t="n"/>
+      <c r="P16" s="23" t="n"/>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="20" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B17" s="21" t="inlineStr">
         <is>
           <t>Shanghai Binyue Trade Co., Ltd.</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C17" s="20" t="inlineStr">
         <is>
           <t>China</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D17" s="22" t="inlineStr">
         <is>
           <t>Shanghai</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E17" s="20" t="inlineStr">
         <is>
           <t>Wholesaler</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F17" s="20" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G17" s="22" t="inlineStr">
         <is>
           <t>Manggis Thailand (merek Limei)</t>
         </is>
       </c>
-      <c r="H11" s="6" t="n"/>
-      <c r="I11" s="7" t="n"/>
-      <c r="J11" s="7" t="n"/>
-      <c r="K11" s="5" t="inlineStr">
+      <c r="H17" s="23" t="n"/>
+      <c r="I17" s="23" t="n"/>
+      <c r="J17" s="23" t="n"/>
+      <c r="K17" s="22" t="inlineStr">
         <is>
           <t>Pasar Buah Huizhan, Shanghai</t>
         </is>
       </c>
-      <c r="L11" s="8" t="inlineStr">
-        <is>
-          <t>https://www.producereport.com/article/thailand-enjoys-lions-share-chinas-mangosteen-market</t>
-        </is>
-      </c>
-      <c r="M11" s="4" t="inlineStr">
-        <is>
-          <t>Tidak ditemukan</t>
-        </is>
-      </c>
-      <c r="N11" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O11" s="9" t="n"/>
-      <c r="P11" s="6" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="n">
+      <c r="L17" s="24" t="inlineStr">
+        <is>
+          <t>producereport.com</t>
+        </is>
+      </c>
+      <c r="M17" s="20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N17" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O17" s="26" t="n"/>
+      <c r="P17" s="23" t="n"/>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B18" s="21" t="inlineStr">
         <is>
           <t>Shanghai Holdfresh Trading Co., Ltd.</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C18" s="20" t="inlineStr">
         <is>
           <t>China</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D18" s="22" t="inlineStr">
         <is>
           <t>Shanghai</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E18" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F18" s="20" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G18" s="22" t="inlineStr">
         <is>
           <t>Buah tropis termasuk manggis</t>
         </is>
       </c>
-      <c r="H12" s="6" t="n"/>
-      <c r="I12" s="7" t="inlineStr">
+      <c r="H18" s="23" t="n"/>
+      <c r="I18" s="23" t="inlineStr">
         <is>
           <t>shanghaiholdfresh@outlook.com</t>
         </is>
       </c>
-      <c r="J12" s="7" t="inlineStr">
+      <c r="J18" s="23" t="inlineStr">
         <is>
           <t>+86 21 6380 6036</t>
         </is>
       </c>
-      <c r="K12" s="5" t="inlineStr">
+      <c r="K18" s="22" t="inlineStr">
         <is>
           <t>Room 270, 2F, Bldg 4, No.130 Huxiang Lane, Sanlin Town, Pudong, Shanghai</t>
         </is>
       </c>
-      <c r="L12" s="8" t="inlineStr">
-        <is>
-          <t>https://www.importgenius.com/importers/shanghai-holdfresh-trading-co-ltd</t>
-        </is>
-      </c>
-      <c r="M12" s="4" t="inlineStr">
+      <c r="L18" s="24" t="inlineStr">
+        <is>
+          <t>importgenius.com</t>
+        </is>
+      </c>
+      <c r="M18" s="20" t="inlineStr">
         <is>
           <t>Sedang</t>
         </is>
       </c>
-      <c r="N12" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O12" s="9" t="n"/>
-      <c r="P12" s="6" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="n">
+      <c r="N18" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O18" s="26" t="n"/>
+      <c r="P18" s="23" t="n"/>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="20" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B19" s="21" t="inlineStr">
         <is>
           <t>Shanghai Sunshine Agriculture Technology Co., Ltd.</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C19" s="20" t="inlineStr">
         <is>
           <t>China</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D19" s="22" t="inlineStr">
         <is>
           <t>Shanghai</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E19" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F19" s="20" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G19" s="22" t="inlineStr">
         <is>
           <t>Manggis dari Indonesia</t>
         </is>
       </c>
-      <c r="H13" s="6" t="n"/>
-      <c r="I13" s="7" t="n"/>
-      <c r="J13" s="7" t="n"/>
-      <c r="K13" s="5" t="inlineStr">
+      <c r="H19" s="23" t="n"/>
+      <c r="I19" s="23" t="n"/>
+      <c r="J19" s="23" t="n"/>
+      <c r="K19" s="22" t="inlineStr">
         <is>
           <t>Room 420-39, No. 1285 Wuwei Road, Putuo District, Shanghai 200331 (belum pasti)</t>
         </is>
       </c>
-      <c r="L13" s="8" t="inlineStr">
-        <is>
-          <t>https://en.nbd.ltd/news/d/668bd591679ff7d42846ca3410eb591e</t>
-        </is>
-      </c>
-      <c r="M13" s="4" t="inlineStr">
+      <c r="L19" s="24" t="inlineStr">
+        <is>
+          <t>en.nbd.ltd</t>
+        </is>
+      </c>
+      <c r="M19" s="20" t="inlineStr">
         <is>
           <t>Sedang</t>
         </is>
       </c>
-      <c r="N13" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O13" s="9" t="n"/>
-      <c r="P13" s="6" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="n">
+      <c r="N19" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O19" s="26" t="n"/>
+      <c r="P19" s="23" t="n"/>
+    </row>
+    <row r="20" ht="47" customHeight="1">
+      <c r="A20" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B20" s="21" t="inlineStr">
         <is>
           <t>CMC Fruit Company Limited</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C20" s="20" t="inlineStr">
         <is>
           <t>Hong Kong</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D20" s="22" t="inlineStr">
         <is>
           <t>Hong Kong</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E20" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F20" s="20" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G20" s="22" t="inlineStr">
         <is>
           <t>Durian, lengkeng, pomelo, longkong Thailand</t>
         </is>
       </c>
-      <c r="H14" s="6" t="n"/>
-      <c r="I14" s="7" t="n"/>
-      <c r="J14" s="7" t="inlineStr">
-        <is>
-          <t>+852 2858 6328; WA +852 9331 1122</t>
-        </is>
-      </c>
-      <c r="K14" s="5" t="inlineStr">
+      <c r="H20" s="23" t="n"/>
+      <c r="I20" s="23" t="n"/>
+      <c r="J20" s="23" t="inlineStr">
+        <is>
+          <t>+852 2858 6328
+WA +852 9331 1122</t>
+        </is>
+      </c>
+      <c r="K20" s="22" t="inlineStr">
         <is>
           <t>Room 3701, 37/F, Chung Kee Commercial Centre, 148 Connaught Road West, Hong Kong</t>
         </is>
       </c>
-      <c r="L14" s="8" t="inlineStr">
-        <is>
-          <t>https://cmcfruit.com/</t>
-        </is>
-      </c>
-      <c r="M14" s="4" t="inlineStr">
+      <c r="L20" s="24" t="inlineStr">
+        <is>
+          <t>cmcfruit.com</t>
+        </is>
+      </c>
+      <c r="M20" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N14" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O14" s="9" t="n"/>
-      <c r="P14" s="6" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="n">
+      <c r="N20" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O20" s="26" t="n"/>
+      <c r="P20" s="23" t="n"/>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="20" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B21" s="21" t="inlineStr">
         <is>
           <t>Sino Alliance Trading (Hong Kong) Limited</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C21" s="20" t="inlineStr">
         <is>
           <t>Hong Kong</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D21" s="22" t="inlineStr">
         <is>
           <t>Yau Ma Tei, Kowloon</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E21" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F21" s="20" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G21" s="22" t="inlineStr">
         <is>
           <t>Buah segar dari 30+ negara</t>
         </is>
       </c>
-      <c r="H15" s="6" t="n"/>
-      <c r="I15" s="7" t="inlineStr">
+      <c r="H21" s="23" t="n"/>
+      <c r="I21" s="23" t="inlineStr">
         <is>
           <t>info@sino-alliance.com</t>
         </is>
       </c>
-      <c r="J15" s="7" t="inlineStr">
+      <c r="J21" s="23" t="inlineStr">
         <is>
           <t>+852 9851 3482</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr">
+      <c r="K21" s="22" t="inlineStr">
         <is>
           <t>Flat 1901, 19/F Bangkok Bank Bldg, 490-492 Nathan Road, Yau Ma Tei, Kowloon, HK</t>
         </is>
       </c>
-      <c r="L15" s="8" t="inlineStr">
-        <is>
-          <t>https://www.sino-alliance.com/en/contact-us/</t>
-        </is>
-      </c>
-      <c r="M15" s="4" t="inlineStr">
+      <c r="L21" s="24" t="inlineStr">
+        <is>
+          <t>sino-alliance.com</t>
+        </is>
+      </c>
+      <c r="M21" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N15" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O15" s="9" t="n"/>
-      <c r="P15" s="6" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="n">
+      <c r="N21" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O21" s="26" t="n"/>
+      <c r="P21" s="23" t="n"/>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="20" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B22" s="21" t="inlineStr">
         <is>
           <t>Joy Wing Mau Fruit Technologies Corp.</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C22" s="20" t="inlineStr">
         <is>
           <t>China</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D22" s="22" t="inlineStr">
         <is>
           <t>Shenzhen</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E22" s="20" t="inlineStr">
         <is>
           <t>Distributor</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F22" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G22" s="22" t="inlineStr">
         <is>
           <t>Buah impor, durian Thailand; distribusi nasional</t>
         </is>
       </c>
-      <c r="H16" s="6" t="n"/>
-      <c r="I16" s="7" t="n"/>
-      <c r="J16" s="7" t="inlineStr">
-        <is>
-          <t>+86 755 2592 8988 / 2518 2988</t>
-        </is>
-      </c>
-      <c r="K16" s="5" t="inlineStr">
+      <c r="H22" s="23" t="n"/>
+      <c r="I22" s="23" t="n"/>
+      <c r="J22" s="23" t="inlineStr">
+        <is>
+          <t>+86 755 2592 8988
+2518 2988</t>
+        </is>
+      </c>
+      <c r="K22" s="22" t="inlineStr">
         <is>
           <t>Joy Wing Mau Binhai Tower, No.170 Hangcheng Avenue, Bao'an, Shenzhen</t>
         </is>
       </c>
-      <c r="L16" s="8" t="inlineStr">
-        <is>
-          <t>https://www.joywingmau.com/homeen/contact/index.html</t>
-        </is>
-      </c>
-      <c r="M16" s="4" t="inlineStr">
+      <c r="L22" s="24" t="inlineStr">
+        <is>
+          <t>joywingmau.com</t>
+        </is>
+      </c>
+      <c r="M22" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N16" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O16" s="9" t="n"/>
-      <c r="P16" s="6" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="n">
+      <c r="N22" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O22" s="26" t="n"/>
+      <c r="P22" s="23" t="n"/>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="20" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B23" s="21" t="inlineStr">
         <is>
           <t>Pagoda (Shenzhen Pagoda Industrial / Baiguoyuan)</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C23" s="20" t="inlineStr">
         <is>
           <t>China</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D23" s="22" t="inlineStr">
         <is>
           <t>Shenzhen</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E23" s="20" t="inlineStr">
         <is>
           <t>Retail/Supermarket</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F23" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G23" s="22" t="inlineStr">
         <is>
           <t>Rantai ritel buah; sourcing langsung luar negeri</t>
         </is>
       </c>
-      <c r="H17" s="6" t="n"/>
-      <c r="I17" s="7" t="n"/>
-      <c r="J17" s="7" t="inlineStr">
-        <is>
-          <t>400-181-1212; +86 755 3686 5476</t>
-        </is>
-      </c>
-      <c r="K17" s="5" t="inlineStr">
+      <c r="H23" s="23" t="n"/>
+      <c r="I23" s="23" t="n"/>
+      <c r="J23" s="23" t="inlineStr">
+        <is>
+          <t>400-181-1212
++86 755 3686 5476</t>
+        </is>
+      </c>
+      <c r="K23" s="22" t="inlineStr">
         <is>
           <t>Baiguoyuan Technology Bldg, No. 2005 Shenyan Road, Haishan Street, Shenzhen</t>
         </is>
       </c>
-      <c r="L17" s="8" t="inlineStr">
-        <is>
-          <t>https://www.pagoda.com.cn/en/about</t>
-        </is>
-      </c>
-      <c r="M17" s="4" t="inlineStr">
+      <c r="L23" s="24" t="inlineStr">
+        <is>
+          <t>pagoda.com.cn</t>
+        </is>
+      </c>
+      <c r="M23" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N17" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O17" s="9" t="n"/>
-      <c r="P17" s="6" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="n">
+      <c r="N23" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O23" s="26" t="n"/>
+      <c r="P23" s="23" t="n"/>
+    </row>
+    <row r="24" ht="34" customHeight="1">
+      <c r="A24" s="20" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B24" s="21" t="inlineStr">
         <is>
           <t>Xianfeng Fruit Co., Ltd.</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C24" s="20" t="inlineStr">
         <is>
           <t>China</t>
         </is>
       </c>
-      <c r="D18" s="4" t="n"/>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="D24" s="22" t="n"/>
+      <c r="E24" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F24" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G24" s="22" t="inlineStr">
         <is>
           <t>Impor global termasuk durian Thailand; punya jaringan toko</t>
         </is>
       </c>
-      <c r="H18" s="6" t="n"/>
-      <c r="I18" s="7" t="n"/>
-      <c r="J18" s="7" t="inlineStr">
+      <c r="H24" s="23" t="n"/>
+      <c r="I24" s="23" t="n"/>
+      <c r="J24" s="23" t="inlineStr">
         <is>
           <t>400 881 9090 (hotline)</t>
         </is>
       </c>
-      <c r="K18" s="5" t="inlineStr">
+      <c r="K24" s="22" t="inlineStr">
         <is>
           <t>No. 85 Sandun Road, Gongshu District, Hangzhou</t>
         </is>
       </c>
-      <c r="L18" s="8" t="inlineStr">
-        <is>
-          <t>http://www.xianfengsg.com/page78</t>
-        </is>
-      </c>
-      <c r="M18" s="4" t="inlineStr">
+      <c r="L24" s="24" t="inlineStr">
+        <is>
+          <t>xianfengsg.com</t>
+        </is>
+      </c>
+      <c r="M24" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N18" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O18" s="9" t="n"/>
-      <c r="P18" s="6" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="n">
+      <c r="N24" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O24" s="26" t="n"/>
+      <c r="P24" s="23" t="n"/>
+    </row>
+    <row r="25" ht="34" customHeight="1">
+      <c r="A25" s="20" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B25" s="21" t="inlineStr">
         <is>
           <t>Bailey Fresh Fruits Co., Ltd. (Prosperity Fresh Fruits Trading)</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C25" s="20" t="inlineStr">
         <is>
           <t>Hong Kong</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D25" s="22" t="inlineStr">
         <is>
           <t>Yau Ma Tei, Kowloon</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E25" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F25" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
+      <c r="G25" s="22" t="inlineStr">
         <is>
           <t>Durian dan buah tropis</t>
         </is>
       </c>
-      <c r="H19" s="6" t="n"/>
-      <c r="I19" s="7" t="n"/>
-      <c r="J19" s="7" t="n"/>
-      <c r="K19" s="5" t="inlineStr">
+      <c r="H25" s="23" t="n"/>
+      <c r="I25" s="23" t="n"/>
+      <c r="J25" s="23" t="n"/>
+      <c r="K25" s="22" t="inlineStr">
         <is>
           <t>G/F 1A Waterloo Road, Yau Ma Tei, Kowloon, HK</t>
         </is>
       </c>
-      <c r="L19" s="8" t="inlineStr">
-        <is>
-          <t>https://panjiva.com/Bailey-Fresh-Fruits-Co-Ltd-T-A-Prosperity-Fresh-Fruits-Trading-Co/149746110</t>
-        </is>
-      </c>
-      <c r="M19" s="4" t="inlineStr">
+      <c r="L25" s="24" t="inlineStr">
+        <is>
+          <t>panjiva.com</t>
+        </is>
+      </c>
+      <c r="M25" s="20" t="inlineStr">
         <is>
           <t>Sedang</t>
         </is>
       </c>
-      <c r="N19" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O19" s="9" t="n"/>
-      <c r="P19" s="6" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="n">
+      <c r="N25" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O25" s="26" t="n"/>
+      <c r="P25" s="23" t="n"/>
+    </row>
+    <row r="26" ht="47" customHeight="1">
+      <c r="A26" s="20" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B26" s="21" t="inlineStr">
         <is>
           <t>Chun Sing Fresh Fruit Trading Limited</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C26" s="20" t="inlineStr">
         <is>
           <t>Hong Kong</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D26" s="22" t="inlineStr">
         <is>
           <t>Yau Ma Tei, Kowloon</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E26" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F26" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G26" s="22" t="inlineStr">
         <is>
           <t>Impor buah &amp; sayur; grosir dan ritel</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="H26" s="23" t="inlineStr">
         <is>
           <t>Tony Lau</t>
         </is>
       </c>
-      <c r="I20" s="7" t="inlineStr">
+      <c r="I26" s="23" t="inlineStr">
         <is>
           <t>chunsingco@gmail.com</t>
         </is>
       </c>
-      <c r="J20" s="7" t="inlineStr">
-        <is>
-          <t>+852 2385 0925; +852 6680 2121 (Tony Lau)</t>
-        </is>
-      </c>
-      <c r="K20" s="5" t="inlineStr">
+      <c r="J26" s="23" t="inlineStr">
+        <is>
+          <t>+852 2385 0925
++852 6680 2121 (Tony Lau)</t>
+        </is>
+      </c>
+      <c r="K26" s="22" t="inlineStr">
         <is>
           <t>No.15 Wholesale Fruit Market, Waterloo Road, Yau Ma Tei, Kowloon, HK</t>
         </is>
       </c>
-      <c r="L20" s="8" t="inlineStr">
-        <is>
-          <t>https://www.csfruit.com.hk/contact</t>
-        </is>
-      </c>
-      <c r="M20" s="4" t="inlineStr">
+      <c r="L26" s="24" t="inlineStr">
+        <is>
+          <t>csfruit.com.hk</t>
+        </is>
+      </c>
+      <c r="M26" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N20" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O20" s="9" t="n"/>
-      <c r="P20" s="6" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="n">
+      <c r="N26" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O26" s="26" t="n"/>
+      <c r="P26" s="23" t="n"/>
+    </row>
+    <row r="27" ht="34" customHeight="1">
+      <c r="A27" s="20" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B27" s="21" t="inlineStr">
         <is>
           <t>Wing Kee Produce Limited</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="C27" s="20" t="inlineStr">
         <is>
           <t>Hong Kong</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D27" s="22" t="inlineStr">
         <is>
           <t>Kowloon Bay</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E27" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="F27" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G21" s="5" t="inlineStr">
+      <c r="G27" s="22" t="inlineStr">
         <is>
           <t>Buah &amp; sayur termasuk tropis</t>
         </is>
       </c>
-      <c r="H21" s="6" t="n"/>
-      <c r="I21" s="7" t="inlineStr">
+      <c r="H27" s="23" t="n"/>
+      <c r="I27" s="23" t="inlineStr">
         <is>
           <t>wkpl@wingkee.com</t>
         </is>
       </c>
-      <c r="J21" s="7" t="inlineStr">
+      <c r="J27" s="23" t="inlineStr">
         <is>
           <t>Sales +852 2796 3111</t>
         </is>
       </c>
-      <c r="K21" s="5" t="inlineStr">
+      <c r="K27" s="22" t="inlineStr">
         <is>
           <t>G/F Hong Leong Ind. Complex, 4 Wang Kwong Road, Kowloon Bay, HK</t>
         </is>
       </c>
-      <c r="L21" s="8" t="inlineStr">
-        <is>
-          <t>https://www.wingkee.com/contact-us/</t>
-        </is>
-      </c>
-      <c r="M21" s="4" t="inlineStr">
+      <c r="L27" s="24" t="inlineStr">
+        <is>
+          <t>wingkee.com</t>
+        </is>
+      </c>
+      <c r="M27" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N21" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O21" s="9" t="n"/>
-      <c r="P21" s="6" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="n">
+      <c r="N27" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O27" s="26" t="n"/>
+      <c r="P27" s="23" t="n"/>
+    </row>
+    <row r="28" ht="47" customHeight="1">
+      <c r="A28" s="20" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B28" s="21" t="inlineStr">
         <is>
           <t>Chongqing Hongjiu Fruit Co., Ltd.</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="C28" s="20" t="inlineStr">
         <is>
           <t>China</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D28" s="22" t="inlineStr">
         <is>
           <t>Chongqing</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E28" s="20" t="inlineStr">
         <is>
           <t>Distributor</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="F28" s="20" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G28" s="22" t="inlineStr">
         <is>
           <t>Durian, manggis, lengkeng Thailand</t>
         </is>
       </c>
-      <c r="H22" s="6" t="n"/>
-      <c r="I22" s="7" t="n"/>
-      <c r="J22" s="7" t="inlineStr">
+      <c r="H28" s="23" t="n"/>
+      <c r="I28" s="23" t="n"/>
+      <c r="J28" s="23" t="inlineStr">
         <is>
           <t>+86 23 6706 4616</t>
         </is>
       </c>
-      <c r="K22" s="5" t="inlineStr">
+      <c r="K28" s="22" t="inlineStr">
         <is>
           <t>22F, Block B, Zhongtiefenghui, No. 3 Donghu South Road, Yubei District, Chongqing</t>
         </is>
       </c>
-      <c r="L22" s="8" t="inlineStr">
-        <is>
-          <t>https://www.hjfruit.com/</t>
-        </is>
-      </c>
-      <c r="M22" s="4" t="inlineStr">
+      <c r="L28" s="24" t="inlineStr">
+        <is>
+          <t>hjfruit.com</t>
+        </is>
+      </c>
+      <c r="M28" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N22" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O22" s="9" t="n"/>
-      <c r="P22" s="6" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="n">
+      <c r="N28" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O28" s="26" t="n"/>
+      <c r="P28" s="23" t="n"/>
+    </row>
+    <row r="29" ht="34" customHeight="1">
+      <c r="A29" s="20" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B29" s="21" t="inlineStr">
         <is>
           <t>Huasheng International Trade (Guangzhou) Co., Ltd.</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="C29" s="20" t="inlineStr">
         <is>
           <t>China</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D29" s="22" t="inlineStr">
         <is>
           <t>Guangzhou</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E29" s="20" t="inlineStr">
         <is>
           <t>Wholesaler</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F29" s="20" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="G29" s="22" t="inlineStr">
         <is>
           <t>Buah impor (ceri, anggur, blueberry, kiwi)</t>
         </is>
       </c>
-      <c r="H23" s="6" t="n"/>
-      <c r="I23" s="7" t="n"/>
-      <c r="J23" s="7" t="n"/>
-      <c r="K23" s="5" t="n"/>
-      <c r="L23" s="8" t="inlineStr">
-        <is>
-          <t>https://www.cnverify.com/company/Huasheng-International-Trade-Guangzhou-Co-Ltd</t>
-        </is>
-      </c>
-      <c r="M23" s="4" t="inlineStr">
-        <is>
-          <t>Tidak ditemukan</t>
-        </is>
-      </c>
-      <c r="N23" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O23" s="9" t="n"/>
-      <c r="P23" s="6" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="n">
+      <c r="H29" s="23" t="n"/>
+      <c r="I29" s="23" t="n"/>
+      <c r="J29" s="23" t="n"/>
+      <c r="K29" s="22" t="n"/>
+      <c r="L29" s="24" t="inlineStr">
+        <is>
+          <t>cnverify.com</t>
+        </is>
+      </c>
+      <c r="M29" s="20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N29" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O29" s="26" t="n"/>
+      <c r="P29" s="23" t="n"/>
+    </row>
+    <row r="30" ht="34" customHeight="1">
+      <c r="A30" s="20" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B30" s="21" t="inlineStr">
         <is>
           <t>Wah Kee Fresh Fruit &amp; Vegetable Ltd</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C30" s="20" t="inlineStr">
         <is>
           <t>Hong Kong</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D30" s="22" t="inlineStr">
         <is>
           <t>Hong Kong</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E30" s="20" t="inlineStr">
         <is>
           <t>Wholesaler</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="F30" s="20" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="G30" s="22" t="inlineStr">
         <is>
           <t>Buah &amp; sayur segar</t>
         </is>
       </c>
-      <c r="H24" s="6" t="n"/>
-      <c r="I24" s="7" t="inlineStr">
+      <c r="H30" s="23" t="n"/>
+      <c r="I30" s="23" t="inlineStr">
         <is>
           <t>wahkeefresh@yahoo.com.hk</t>
         </is>
       </c>
-      <c r="J24" s="7" t="inlineStr">
+      <c r="J30" s="23" t="inlineStr">
         <is>
           <t>+852 2545 7182</t>
         </is>
       </c>
-      <c r="K24" s="5" t="inlineStr">
+      <c r="K30" s="22" t="inlineStr">
         <is>
           <t>Stall C120, Western Wholesale Food Market, 8 Fung Mat Rd, Sai Wan, HK</t>
         </is>
       </c>
-      <c r="L24" s="8" t="inlineStr">
-        <is>
-          <t>https://sourcing.hktdc.com/en/Supplier-Store-Directory/Wah-Kee-Fresh-Fruit-Vegetable-Ltd/1X09P9CX</t>
-        </is>
-      </c>
-      <c r="M24" s="4" t="inlineStr">
+      <c r="L30" s="24" t="inlineStr">
+        <is>
+          <t>sourcing.hktdc.com</t>
+        </is>
+      </c>
+      <c r="M30" s="20" t="inlineStr">
         <is>
           <t>Sedang</t>
         </is>
       </c>
-      <c r="N24" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O24" s="9" t="n"/>
-      <c r="P24" s="6" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="n">
+      <c r="N30" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O30" s="26" t="n"/>
+      <c r="P30" s="23" t="n"/>
+    </row>
+    <row r="31" ht="47" customHeight="1">
+      <c r="A31" s="20" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B31" s="21" t="inlineStr">
         <is>
           <t>Al Yusra Foodstuff Trading LLC</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C31" s="20" t="inlineStr">
         <is>
           <t>UAE</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D31" s="22" t="inlineStr">
         <is>
           <t>Dubai</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E31" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F31" s="20" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="G31" s="22" t="inlineStr">
         <is>
           <t>Importir, distributor, commission agent buah &amp; sayur; lini eksotis</t>
         </is>
       </c>
-      <c r="H25" s="6" t="n"/>
-      <c r="I25" s="7" t="n"/>
-      <c r="J25" s="7" t="inlineStr">
+      <c r="H31" s="23" t="n"/>
+      <c r="I31" s="23" t="n"/>
+      <c r="J31" s="23" t="inlineStr">
         <is>
           <t>+971 56 180 7028</t>
         </is>
       </c>
-      <c r="K25" s="5" t="inlineStr">
+      <c r="K31" s="22" t="inlineStr">
         <is>
           <t>Office 20, GF, Khalifa Bldg, Street 14, Abu Hail, Dubai</t>
         </is>
       </c>
-      <c r="L25" s="8" t="inlineStr">
-        <is>
-          <t>https://www.alyusrafoodstuff.com/contact-us.php</t>
-        </is>
-      </c>
-      <c r="M25" s="4" t="inlineStr">
+      <c r="L31" s="24" t="inlineStr">
+        <is>
+          <t>alyusrafoodstuff.com</t>
+        </is>
+      </c>
+      <c r="M31" s="20" t="inlineStr">
         <is>
           <t>Sedang</t>
         </is>
       </c>
-      <c r="N25" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O25" s="9" t="n"/>
-      <c r="P25" s="6" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="n">
+      <c r="N31" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O31" s="26" t="n"/>
+      <c r="P31" s="23" t="n"/>
+    </row>
+    <row r="32" ht="34" customHeight="1">
+      <c r="A32" s="20" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B32" s="21" t="inlineStr">
         <is>
           <t>Anusaya Fresh (Anusuya Fresh Fruits &amp; Vegetables LLC)</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C32" s="20" t="inlineStr">
         <is>
           <t>UAE</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D32" s="22" t="inlineStr">
         <is>
           <t>Dubai (Al Aweer)</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E32" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="F32" s="20" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="G32" s="22" t="inlineStr">
         <is>
           <t>Apel, jeruk, anggur + eksotis: manggis, rambutan, buah naga</t>
         </is>
       </c>
-      <c r="H26" s="6" t="n"/>
-      <c r="I26" s="7" t="inlineStr">
+      <c r="H32" s="23" t="n"/>
+      <c r="I32" s="23" t="inlineStr">
         <is>
           <t>salesdxb@anusayafresh.com</t>
         </is>
       </c>
-      <c r="J26" s="7" t="n"/>
-      <c r="K26" s="5" t="inlineStr">
+      <c r="J32" s="23" t="n"/>
+      <c r="K32" s="22" t="inlineStr">
         <is>
           <t>Al Asmawi Warehouses, Warehouse No. 8, P.O. Box 10166, Al Aweer, Dubai</t>
         </is>
       </c>
-      <c r="L26" s="8" t="inlineStr">
-        <is>
-          <t>http://www.anusayafresh.com/contact.html</t>
-        </is>
-      </c>
-      <c r="M26" s="4" t="inlineStr">
+      <c r="L32" s="24" t="inlineStr">
+        <is>
+          <t>anusayafresh.com</t>
+        </is>
+      </c>
+      <c r="M32" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N26" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O26" s="9" t="n"/>
-      <c r="P26" s="6" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="n">
+      <c r="N32" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O32" s="26" t="n"/>
+      <c r="P32" s="23" t="n"/>
+    </row>
+    <row r="33" ht="34" customHeight="1">
+      <c r="A33" s="20" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B33" s="21" t="inlineStr">
         <is>
           <t>Euto Foods Trading</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="C33" s="20" t="inlineStr">
         <is>
           <t>UAE</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D33" s="22" t="inlineStr">
         <is>
           <t>Dubai</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="E33" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="F33" s="20" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
+      <c r="G33" s="22" t="inlineStr">
         <is>
           <t>Importir buah grosir; tropis termasuk manggis</t>
         </is>
       </c>
-      <c r="H27" s="6" t="n"/>
-      <c r="I27" s="7" t="n"/>
-      <c r="J27" s="7" t="n"/>
-      <c r="K27" s="5" t="n"/>
-      <c r="L27" s="8" t="inlineStr">
-        <is>
-          <t>https://eutofoods.com/</t>
-        </is>
-      </c>
-      <c r="M27" s="4" t="inlineStr">
-        <is>
-          <t>Tidak ditemukan</t>
-        </is>
-      </c>
-      <c r="N27" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O27" s="9" t="n"/>
-      <c r="P27" s="6" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="n">
+      <c r="H33" s="23" t="n"/>
+      <c r="I33" s="23" t="n"/>
+      <c r="J33" s="23" t="n"/>
+      <c r="K33" s="22" t="n"/>
+      <c r="L33" s="24" t="inlineStr">
+        <is>
+          <t>eutofoods.com</t>
+        </is>
+      </c>
+      <c r="M33" s="20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N33" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O33" s="26" t="n"/>
+      <c r="P33" s="23" t="n"/>
+    </row>
+    <row r="34" ht="34" customHeight="1">
+      <c r="A34" s="20" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B34" s="21" t="inlineStr">
         <is>
           <t>Fresh Leaf UAE</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="C34" s="20" t="inlineStr">
         <is>
           <t>UAE</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D34" s="22" t="inlineStr">
         <is>
           <t>Dubai</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E34" s="20" t="inlineStr">
         <is>
           <t>Distributor</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="F34" s="20" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="G34" s="22" t="inlineStr">
         <is>
           <t>Kategori buah eksotis termasuk 'Mangosteen Indonesia'</t>
         </is>
       </c>
-      <c r="H28" s="6" t="n"/>
-      <c r="I28" s="7" t="n"/>
-      <c r="J28" s="7" t="inlineStr">
+      <c r="H34" s="23" t="n"/>
+      <c r="I34" s="23" t="n"/>
+      <c r="J34" s="23" t="inlineStr">
         <is>
           <t>+971 55 446 6860</t>
         </is>
       </c>
-      <c r="K28" s="5" t="inlineStr">
+      <c r="K34" s="22" t="inlineStr">
         <is>
           <t>Shop #13, Block #12, Fruits &amp; Vegetables Market, Al Aweer, Dubai</t>
         </is>
       </c>
-      <c r="L28" s="8" t="inlineStr">
-        <is>
-          <t>https://freshleafuae.com/contact/</t>
-        </is>
-      </c>
-      <c r="M28" s="4" t="inlineStr">
+      <c r="L34" s="24" t="inlineStr">
+        <is>
+          <t>freshleafuae.com</t>
+        </is>
+      </c>
+      <c r="M34" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N28" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O28" s="9" t="n"/>
-      <c r="P28" s="6" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="n">
+      <c r="N34" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O34" s="26" t="n"/>
+      <c r="P34" s="23" t="n"/>
+    </row>
+    <row r="35" ht="34" customHeight="1">
+      <c r="A35" s="20" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B35" s="21" t="inlineStr">
         <is>
           <t>Source International</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C35" s="20" t="inlineStr">
         <is>
           <t>UAE</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D35" s="22" t="inlineStr">
         <is>
           <t>Dubai</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E35" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="F35" s="20" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr">
+      <c r="G35" s="22" t="inlineStr">
         <is>
           <t>Importir/distributor buah eksotis B2B</t>
         </is>
       </c>
-      <c r="H29" s="6" t="n"/>
-      <c r="I29" s="7" t="inlineStr">
+      <c r="H35" s="23" t="n"/>
+      <c r="I35" s="23" t="inlineStr">
         <is>
           <t>info@sourceinternational.ae</t>
         </is>
       </c>
-      <c r="J29" s="7" t="inlineStr">
-        <is>
-          <t>+971 50 664 3592; +971 54 440 7354</t>
-        </is>
-      </c>
-      <c r="K29" s="5" t="n"/>
-      <c r="L29" s="8" t="inlineStr">
-        <is>
-          <t>https://sourceinternational.ae/contact/</t>
-        </is>
-      </c>
-      <c r="M29" s="4" t="inlineStr">
+      <c r="J35" s="23" t="inlineStr">
+        <is>
+          <t>+971 50 664 3592
++971 54 440 7354</t>
+        </is>
+      </c>
+      <c r="K35" s="22" t="n"/>
+      <c r="L35" s="24" t="inlineStr">
+        <is>
+          <t>sourceinternational.ae</t>
+        </is>
+      </c>
+      <c r="M35" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N29" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O29" s="9" t="n"/>
-      <c r="P29" s="6" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="n">
+      <c r="N35" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O35" s="26" t="n"/>
+      <c r="P35" s="23" t="n"/>
+    </row>
+    <row r="36" ht="34" customHeight="1">
+      <c r="A36" s="20" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B36" s="21" t="inlineStr">
         <is>
           <t>AlQatari Fruits Company W.L.L.</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="C36" s="20" t="inlineStr">
         <is>
           <t>Bahrain</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D36" s="22" t="inlineStr">
         <is>
           <t>Manama</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E36" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="F36" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr">
+      <c r="G36" s="22" t="inlineStr">
         <is>
           <t>Impor, re-ekspor, grosir buah &amp; sayur sejak 1943</t>
         </is>
       </c>
-      <c r="H30" s="6" t="n"/>
-      <c r="I30" s="7" t="inlineStr">
-        <is>
-          <t>alqatarifruits@batelco.com.bh; alqatarifruit@gmail.com</t>
-        </is>
-      </c>
-      <c r="J30" s="7" t="n"/>
-      <c r="K30" s="5" t="inlineStr">
+      <c r="H36" s="23" t="n"/>
+      <c r="I36" s="23" t="inlineStr">
+        <is>
+          <t>alqatarifruits@batelco.com.bh
+alqatarifruit@gmail.com</t>
+        </is>
+      </c>
+      <c r="J36" s="23" t="n"/>
+      <c r="K36" s="22" t="inlineStr">
         <is>
           <t>51 Block 314, Street 1404, Manama, Bahrain</t>
         </is>
       </c>
-      <c r="L30" s="8" t="inlineStr">
-        <is>
-          <t>https://www.alqatarifruits.com/contacts.html</t>
-        </is>
-      </c>
-      <c r="M30" s="4" t="inlineStr">
+      <c r="L36" s="24" t="inlineStr">
+        <is>
+          <t>alqatarifruits.com</t>
+        </is>
+      </c>
+      <c r="M36" s="20" t="inlineStr">
         <is>
           <t>Sedang</t>
         </is>
       </c>
-      <c r="N30" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O30" s="9" t="n"/>
-      <c r="P30" s="6" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="n">
+      <c r="N36" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O36" s="26" t="n"/>
+      <c r="P36" s="23" t="n"/>
+    </row>
+    <row r="37" ht="34" customHeight="1">
+      <c r="A37" s="20" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B37" s="21" t="inlineStr">
         <is>
           <t>Suma Fruits International Co. WLL</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="C37" s="20" t="inlineStr">
         <is>
           <t>Kuwait</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D37" s="22" t="inlineStr">
         <is>
           <t>Kuwait City (Ardhiya)</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="E37" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="F37" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="G37" s="22" t="inlineStr">
         <is>
           <t>Nanas, mangga, plum; asal Filipina/Vietnam/Sri Lanka</t>
         </is>
       </c>
-      <c r="H31" s="6" t="n"/>
-      <c r="I31" s="7" t="n"/>
-      <c r="J31" s="7" t="inlineStr">
+      <c r="H37" s="23" t="n"/>
+      <c r="I37" s="23" t="n"/>
+      <c r="J37" s="23" t="inlineStr">
         <is>
           <t>+965 2226 6880</t>
         </is>
       </c>
-      <c r="K31" s="5" t="n"/>
-      <c r="L31" s="8" t="inlineStr">
-        <is>
-          <t>https://sumafruits.com/en/contactus</t>
-        </is>
-      </c>
-      <c r="M31" s="4" t="inlineStr">
+      <c r="K37" s="22" t="n"/>
+      <c r="L37" s="24" t="inlineStr">
+        <is>
+          <t>sumafruits.com</t>
+        </is>
+      </c>
+      <c r="M37" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N31" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O31" s="9" t="n"/>
-      <c r="P31" s="6" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="n">
+      <c r="N37" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O37" s="26" t="n"/>
+      <c r="P37" s="23" t="n"/>
+    </row>
+    <row r="38" ht="34" customHeight="1">
+      <c r="A38" s="20" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B38" s="21" t="inlineStr">
         <is>
           <t>Al Shahabi Trading Co.</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C38" s="20" t="inlineStr">
         <is>
           <t>Qatar</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D38" s="22" t="inlineStr">
         <is>
           <t>Doha</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="E38" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="F38" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G32" s="5" t="inlineStr">
+      <c r="G38" s="22" t="inlineStr">
         <is>
           <t>Importir buah &amp; sayur, salah satu tertua di Qatar</t>
         </is>
       </c>
-      <c r="H32" s="6" t="inlineStr">
+      <c r="H38" s="23" t="inlineStr">
         <is>
           <t>Mr. Ebrahim Alshahabi</t>
         </is>
       </c>
-      <c r="I32" s="7" t="inlineStr">
+      <c r="I38" s="23" t="inlineStr">
         <is>
           <t>e.shahabi@alshahabifruits.com</t>
         </is>
       </c>
-      <c r="J32" s="7" t="inlineStr">
+      <c r="J38" s="23" t="inlineStr">
         <is>
           <t>+974 4468 6557</t>
         </is>
       </c>
-      <c r="K32" s="5" t="inlineStr">
+      <c r="K38" s="22" t="inlineStr">
         <is>
           <t>P.O. Box 5405, Logistic Park A, Al Wakra, Qatar</t>
         </is>
       </c>
-      <c r="L32" s="8" t="inlineStr">
-        <is>
-          <t>https://alshahabifruits.com/</t>
-        </is>
-      </c>
-      <c r="M32" s="4" t="inlineStr">
+      <c r="L38" s="24" t="inlineStr">
+        <is>
+          <t>alshahabifruits.com</t>
+        </is>
+      </c>
+      <c r="M38" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N32" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O32" s="9" t="n"/>
-      <c r="P32" s="6" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="n">
+      <c r="N38" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O38" s="26" t="n"/>
+      <c r="P38" s="23" t="n"/>
+    </row>
+    <row r="39" ht="34" customHeight="1">
+      <c r="A39" s="20" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B39" s="21" t="inlineStr">
         <is>
           <t>Royal Fresh Fruits</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C39" s="20" t="inlineStr">
         <is>
           <t>Qatar</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D39" s="22" t="inlineStr">
         <is>
           <t>Doha</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="E39" s="20" t="inlineStr">
         <is>
           <t>Wholesaler</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="F39" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G33" s="5" t="inlineStr">
+      <c r="G39" s="22" t="inlineStr">
         <is>
           <t>Importir/grosir dari Eropa, Asia, Afrika, Australia</t>
         </is>
       </c>
-      <c r="H33" s="6" t="n"/>
-      <c r="I33" s="7" t="inlineStr">
+      <c r="H39" s="23" t="n"/>
+      <c r="I39" s="23" t="inlineStr">
         <is>
           <t>info@rff.qa</t>
         </is>
       </c>
-      <c r="J33" s="7" t="n"/>
-      <c r="K33" s="5" t="inlineStr">
+      <c r="J39" s="23" t="n"/>
+      <c r="K39" s="22" t="inlineStr">
         <is>
           <t>Industrial Area Street 37 &amp; Street 52, Doha, Qatar</t>
         </is>
       </c>
-      <c r="L33" s="8" t="inlineStr">
-        <is>
-          <t>https://rff.qa/</t>
-        </is>
-      </c>
-      <c r="M33" s="4" t="inlineStr">
-        <is>
-          <t>Tinggi (alamat), Sedang (email)</t>
-        </is>
-      </c>
-      <c r="N33" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O33" s="9" t="n"/>
-      <c r="P33" s="6" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="4" t="n">
+      <c r="L39" s="24" t="inlineStr">
+        <is>
+          <t>rff.qa</t>
+        </is>
+      </c>
+      <c r="M39" s="20" t="inlineStr">
+        <is>
+          <t>Tinggi</t>
+        </is>
+      </c>
+      <c r="N39" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O39" s="26" t="n"/>
+      <c r="P39" s="23" t="n"/>
+    </row>
+    <row r="40" ht="34" customHeight="1">
+      <c r="A40" s="20" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B40" s="21" t="inlineStr">
         <is>
           <t>World Fruits Centre</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="C40" s="20" t="inlineStr">
         <is>
           <t>Qatar</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D40" s="22" t="inlineStr">
         <is>
           <t>Doha</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E40" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="F40" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G34" s="5" t="inlineStr">
+      <c r="G40" s="22" t="inlineStr">
         <is>
           <t>Importir buah &amp; sayur untuk hotel, food service, supermarket</t>
         </is>
       </c>
-      <c r="H34" s="6" t="n"/>
-      <c r="I34" s="7" t="inlineStr">
+      <c r="H40" s="23" t="n"/>
+      <c r="I40" s="23" t="inlineStr">
         <is>
           <t>info@wfc-qatar.com</t>
         </is>
       </c>
-      <c r="J34" s="7" t="inlineStr">
-        <is>
-          <t>+974 4469 7714 / 4468 2285</t>
-        </is>
-      </c>
-      <c r="K34" s="5" t="inlineStr">
+      <c r="J40" s="23" t="inlineStr">
+        <is>
+          <t>+974 4469 7714
+4468 2285</t>
+        </is>
+      </c>
+      <c r="K40" s="22" t="inlineStr">
         <is>
           <t>PO Box 9427, Um Sulal Ali, Doha, Qatar</t>
         </is>
       </c>
-      <c r="L34" s="8" t="inlineStr">
-        <is>
-          <t>https://www.wfc-qatar.com/</t>
-        </is>
-      </c>
-      <c r="M34" s="4" t="inlineStr">
+      <c r="L40" s="24" t="inlineStr">
+        <is>
+          <t>wfc-qatar.com</t>
+        </is>
+      </c>
+      <c r="M40" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N34" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O34" s="9" t="n"/>
-      <c r="P34" s="6" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="n">
+      <c r="N40" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O40" s="26" t="n"/>
+      <c r="P40" s="23" t="n"/>
+    </row>
+    <row r="41" ht="34" customHeight="1">
+      <c r="A41" s="20" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B41" s="21" t="inlineStr">
         <is>
           <t>AFDAN Company for Fruits and Vegetables Trading</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C41" s="20" t="inlineStr">
         <is>
           <t>Saudi Arabia</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D41" s="22" t="inlineStr">
         <is>
           <t>Riyadh</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="E41" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="F41" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G35" s="5" t="inlineStr">
+      <c r="G41" s="22" t="inlineStr">
         <is>
           <t>Pengadaan/impor global buah &amp; sayur</t>
         </is>
       </c>
-      <c r="H35" s="6" t="n"/>
-      <c r="I35" s="7" t="inlineStr">
+      <c r="H41" s="23" t="n"/>
+      <c r="I41" s="23" t="inlineStr">
         <is>
           <t>info@afdan.sa</t>
         </is>
       </c>
-      <c r="J35" s="7" t="inlineStr">
+      <c r="J41" s="23" t="inlineStr">
         <is>
           <t>+966 50 537 8670</t>
         </is>
       </c>
-      <c r="K35" s="5" t="inlineStr">
+      <c r="K41" s="22" t="inlineStr">
         <is>
           <t>Riyadh, Saudi Arabia</t>
         </is>
       </c>
-      <c r="L35" s="8" t="inlineStr">
-        <is>
-          <t>https://www.afdan.sa/en/contact-us.php</t>
-        </is>
-      </c>
-      <c r="M35" s="4" t="inlineStr">
+      <c r="L41" s="24" t="inlineStr">
+        <is>
+          <t>afdan.sa</t>
+        </is>
+      </c>
+      <c r="M41" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N35" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O35" s="9" t="n"/>
-      <c r="P35" s="6" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="n">
+      <c r="N41" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O41" s="26" t="n"/>
+      <c r="P41" s="23" t="n"/>
+    </row>
+    <row r="42" ht="47" customHeight="1">
+      <c r="A42" s="20" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B42" s="21" t="inlineStr">
         <is>
           <t>BlissBerrys</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="C42" s="20" t="inlineStr">
         <is>
           <t>Saudi Arabia</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D42" s="22" t="inlineStr">
         <is>
           <t>Riyadh/Jeddah/Dammam</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="E42" s="20" t="inlineStr">
         <is>
           <t>Distributor</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
+      <c r="F42" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G36" s="5" t="inlineStr">
+      <c r="G42" s="22" t="inlineStr">
         <is>
           <t>Alpukat, mangga, nanas, beri, jeruk ke supermarket &amp; HoReCa</t>
         </is>
       </c>
-      <c r="H36" s="6" t="n"/>
-      <c r="I36" s="7" t="inlineStr">
+      <c r="H42" s="23" t="n"/>
+      <c r="I42" s="23" t="inlineStr">
         <is>
           <t>Office@blissberrys.com</t>
         </is>
       </c>
-      <c r="J36" s="7" t="inlineStr">
-        <is>
-          <t>+966 11 269 7137; +966 55 029 7817; +966 55 097 4991</t>
-        </is>
-      </c>
-      <c r="K36" s="5" t="n"/>
-      <c r="L36" s="8" t="inlineStr">
-        <is>
-          <t>https://blissberrys.com/contact-blissberry-fruit-vegetable-supplier/</t>
-        </is>
-      </c>
-      <c r="M36" s="4" t="inlineStr">
+      <c r="J42" s="23" t="inlineStr">
+        <is>
+          <t>+966 11 269 7137
++966 55 029 7817
++966 55 097 4991</t>
+        </is>
+      </c>
+      <c r="K42" s="22" t="n"/>
+      <c r="L42" s="24" t="inlineStr">
+        <is>
+          <t>blissberrys.com</t>
+        </is>
+      </c>
+      <c r="M42" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N36" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O36" s="9" t="n"/>
-      <c r="P36" s="6" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="4" t="n">
+      <c r="N42" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O42" s="26" t="n"/>
+      <c r="P42" s="23" t="n"/>
+    </row>
+    <row r="43" ht="34" customHeight="1">
+      <c r="A43" s="20" t="n">
         <v>33</v>
       </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B43" s="21" t="inlineStr">
         <is>
           <t>Sharbatly Fruit</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C43" s="20" t="inlineStr">
         <is>
           <t>Saudi Arabia</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D43" s="22" t="inlineStr">
         <is>
           <t>Jeddah</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="E43" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr">
+      <c r="F43" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G37" s="5" t="inlineStr">
+      <c r="G43" s="22" t="inlineStr">
         <is>
           <t>Importir/distributor produk segar premium sejak 1930-an</t>
         </is>
       </c>
-      <c r="H37" s="6" t="n"/>
-      <c r="I37" s="7" t="inlineStr">
+      <c r="H43" s="23" t="n"/>
+      <c r="I43" s="23" t="inlineStr">
         <is>
           <t>info@sharbatly.com</t>
         </is>
       </c>
-      <c r="J37" s="7" t="inlineStr">
+      <c r="J43" s="23" t="inlineStr">
         <is>
           <t>+966 12 679 0000</t>
         </is>
       </c>
-      <c r="K37" s="5" t="n"/>
-      <c r="L37" s="8" t="inlineStr">
-        <is>
-          <t>https://www.sharbatlyfruit.com/en/contact-us</t>
-        </is>
-      </c>
-      <c r="M37" s="4" t="inlineStr">
+      <c r="K43" s="22" t="n"/>
+      <c r="L43" s="24" t="inlineStr">
+        <is>
+          <t>sharbatlyfruit.com</t>
+        </is>
+      </c>
+      <c r="M43" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N37" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O37" s="9" t="n"/>
-      <c r="P37" s="6" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="n">
+      <c r="N43" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O43" s="26" t="n"/>
+      <c r="P43" s="23" t="n"/>
+    </row>
+    <row r="44" ht="34" customHeight="1">
+      <c r="A44" s="20" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="5" t="inlineStr">
+      <c r="B44" s="21" t="inlineStr">
         <is>
           <t>Shrayan Al Jazeera Fruits &amp; Vegetables Trading</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="C44" s="20" t="inlineStr">
         <is>
           <t>Saudi Arabia</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D44" s="22" t="inlineStr">
         <is>
           <t>Jeddah</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="E44" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="F44" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G38" s="5" t="inlineStr">
+      <c r="G44" s="22" t="inlineStr">
         <is>
           <t>Impor/ekspor buah &amp; sayur sejak 2009</t>
         </is>
       </c>
-      <c r="H38" s="6" t="n"/>
-      <c r="I38" s="7" t="inlineStr">
+      <c r="H44" s="23" t="n"/>
+      <c r="I44" s="23" t="inlineStr">
         <is>
           <t>info@shrayanaljazeera.com</t>
         </is>
       </c>
-      <c r="J38" s="7" t="n"/>
-      <c r="K38" s="5" t="inlineStr">
+      <c r="J44" s="23" t="n"/>
+      <c r="K44" s="22" t="inlineStr">
         <is>
           <t>Panorama Centre, Office 5, Umm Al Qura Street, Safa, Jeddah, Saudi Arabia</t>
         </is>
       </c>
-      <c r="L38" s="8" t="inlineStr">
-        <is>
-          <t>https://shrayanaljazeera.com/contact/</t>
-        </is>
-      </c>
-      <c r="M38" s="4" t="inlineStr">
+      <c r="L44" s="24" t="inlineStr">
+        <is>
+          <t>shrayanaljazeera.com</t>
+        </is>
+      </c>
+      <c r="M44" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N38" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O38" s="9" t="n"/>
-      <c r="P38" s="6" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="n">
+      <c r="N44" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O44" s="26" t="n"/>
+      <c r="P44" s="23" t="n"/>
+    </row>
+    <row r="45" ht="47" customHeight="1">
+      <c r="A45" s="20" t="n">
         <v>35</v>
       </c>
-      <c r="B39" s="5" t="inlineStr">
+      <c r="B45" s="21" t="inlineStr">
         <is>
           <t>AJMEER General Trading LLC</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C45" s="20" t="inlineStr">
         <is>
           <t>UAE</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D45" s="22" t="inlineStr">
         <is>
           <t>Dubai (Al Aweer)</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="E45" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr">
+      <c r="F45" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G39" s="5" t="inlineStr">
+      <c r="G45" s="22" t="inlineStr">
         <is>
           <t>Impor buah &amp; sayur dari Asia, Eropa, Afrika; suplai hotel &amp; ritel</t>
         </is>
       </c>
-      <c r="H39" s="6" t="n"/>
-      <c r="I39" s="7" t="inlineStr">
+      <c r="H45" s="23" t="n"/>
+      <c r="I45" s="23" t="inlineStr">
         <is>
           <t>mail@ajmeer.ae</t>
         </is>
       </c>
-      <c r="J39" s="7" t="inlineStr">
+      <c r="J45" s="23" t="inlineStr">
         <is>
           <t>+971 4 438 5061</t>
         </is>
       </c>
-      <c r="K39" s="5" t="inlineStr">
+      <c r="K45" s="22" t="inlineStr">
         <is>
           <t>Al Aweer Central Fruits &amp; Vegetables Market; P.O. Box 234276, Dubai</t>
         </is>
       </c>
-      <c r="L39" s="8" t="inlineStr">
-        <is>
-          <t>https://ajmeer.ae/contact-us/</t>
-        </is>
-      </c>
-      <c r="M39" s="4" t="inlineStr">
+      <c r="L45" s="24" t="inlineStr">
+        <is>
+          <t>ajmeer.ae</t>
+        </is>
+      </c>
+      <c r="M45" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N39" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O39" s="9" t="n"/>
-      <c r="P39" s="6" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="4" t="n">
+      <c r="N45" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O45" s="26" t="n"/>
+      <c r="P45" s="23" t="n"/>
+    </row>
+    <row r="46" ht="47" customHeight="1">
+      <c r="A46" s="20" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="5" t="inlineStr">
+      <c r="B46" s="21" t="inlineStr">
         <is>
           <t>Barakat Vegetables &amp; Fruits Co. LLC</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="C46" s="20" t="inlineStr">
         <is>
           <t>UAE</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D46" s="22" t="inlineStr">
         <is>
           <t>Dubai (Al Aweer)</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
+      <c r="E46" s="20" t="inlineStr">
         <is>
           <t>Distributor</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr">
+      <c r="F46" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G40" s="5" t="inlineStr">
+      <c r="G46" s="22" t="inlineStr">
         <is>
           <t>Importir/distributor besar (53+ negara asal); HoReCa, ritel</t>
         </is>
       </c>
-      <c r="H40" s="6" t="n"/>
-      <c r="I40" s="7" t="inlineStr">
+      <c r="H46" s="23" t="n"/>
+      <c r="I46" s="23" t="inlineStr">
         <is>
           <t>contact@barakatuae.ae</t>
         </is>
       </c>
-      <c r="J40" s="7" t="inlineStr">
+      <c r="J46" s="23" t="inlineStr">
         <is>
           <t>800 2272 528</t>
         </is>
       </c>
-      <c r="K40" s="5" t="inlineStr">
+      <c r="K46" s="22" t="inlineStr">
         <is>
           <t>Shop 27/A, Wholesale Bldg 2, Central Fruits &amp; Vegetables Market, Al Aweer, PO Box 11286, Dubai</t>
         </is>
       </c>
-      <c r="L40" s="8" t="inlineStr">
-        <is>
-          <t>http://www.barakatgroup.ae/contact.php</t>
-        </is>
-      </c>
-      <c r="M40" s="4" t="inlineStr">
+      <c r="L46" s="24" t="inlineStr">
+        <is>
+          <t>barakatgroup.ae</t>
+        </is>
+      </c>
+      <c r="M46" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N40" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O40" s="9" t="n"/>
-      <c r="P40" s="6" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="4" t="n">
+      <c r="N46" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O46" s="26" t="n"/>
+      <c r="P46" s="23" t="n"/>
+    </row>
+    <row r="47" ht="34" customHeight="1">
+      <c r="A47" s="20" t="n">
         <v>37</v>
       </c>
-      <c r="B41" s="5" t="inlineStr">
+      <c r="B47" s="21" t="inlineStr">
         <is>
           <t>Fresh Avenue Foodstuff Trading LLC</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C47" s="20" t="inlineStr">
         <is>
           <t>UAE</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D47" s="22" t="inlineStr">
         <is>
           <t>Dubai (Al Aweer)</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="E47" s="20" t="inlineStr">
         <is>
           <t>Wholesaler</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr">
+      <c r="F47" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G41" s="5" t="inlineStr">
+      <c r="G47" s="22" t="inlineStr">
         <is>
           <t>Grosir buah &amp; sayur, termasuk rambutan</t>
         </is>
       </c>
-      <c r="H41" s="6" t="n"/>
-      <c r="I41" s="7" t="inlineStr">
+      <c r="H47" s="23" t="n"/>
+      <c r="I47" s="23" t="inlineStr">
         <is>
           <t>freshavenue.dxb@gmail.com</t>
         </is>
       </c>
-      <c r="J41" s="7" t="inlineStr">
-        <is>
-          <t>+971 54 177 0064; +971 54 181 3596</t>
-        </is>
-      </c>
-      <c r="K41" s="5" t="inlineStr">
+      <c r="J47" s="23" t="inlineStr">
+        <is>
+          <t>+971 54 177 0064
++971 54 181 3596</t>
+        </is>
+      </c>
+      <c r="K47" s="22" t="inlineStr">
         <is>
           <t>Al Aweer Central Fruit &amp; Vegetable Market, Dubai</t>
         </is>
       </c>
-      <c r="L41" s="8" t="inlineStr">
-        <is>
-          <t>https://www.freshavenuefoodstufftradingllc.com/</t>
-        </is>
-      </c>
-      <c r="M41" s="4" t="inlineStr">
+      <c r="L47" s="24" t="inlineStr">
+        <is>
+          <t>freshavenuefoodstufftradingllc.com</t>
+        </is>
+      </c>
+      <c r="M47" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N41" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O41" s="9" t="n"/>
-      <c r="P41" s="6" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="4" t="n">
+      <c r="N47" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O47" s="26" t="n"/>
+      <c r="P47" s="23" t="n"/>
+    </row>
+    <row r="48" ht="34" customHeight="1">
+      <c r="A48" s="20" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="5" t="inlineStr">
+      <c r="B48" s="21" t="inlineStr">
         <is>
           <t>Kibsons</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
+      <c r="C48" s="20" t="inlineStr">
         <is>
           <t>UAE</t>
         </is>
       </c>
-      <c r="D42" s="4" t="inlineStr">
+      <c r="D48" s="22" t="inlineStr">
         <is>
           <t>Dubai (Al Aweer)</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
+      <c r="E48" s="20" t="inlineStr">
         <is>
           <t>E-commerce</t>
         </is>
       </c>
-      <c r="F42" s="4" t="inlineStr">
+      <c r="F48" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G42" s="5" t="inlineStr">
+      <c r="G48" s="22" t="inlineStr">
         <is>
           <t>Grocery online dengan kategori buah eksotis</t>
         </is>
       </c>
-      <c r="H42" s="6" t="n"/>
-      <c r="I42" s="7" t="inlineStr">
+      <c r="H48" s="23" t="n"/>
+      <c r="I48" s="23" t="inlineStr">
         <is>
           <t>customercare@kibsons.com</t>
         </is>
       </c>
-      <c r="J42" s="7" t="inlineStr">
+      <c r="J48" s="23" t="inlineStr">
         <is>
           <t>800 KIBSONS (800 5427667)</t>
         </is>
       </c>
-      <c r="K42" s="5" t="inlineStr">
+      <c r="K48" s="22" t="inlineStr">
         <is>
           <t>Manama Street, Ras Al Khor 2, Dubai; PO Box 5313, Dubai, UAE</t>
         </is>
       </c>
-      <c r="L42" s="8" t="inlineStr">
-        <is>
-          <t>https://www.kibsons.com/en/contactus</t>
-        </is>
-      </c>
-      <c r="M42" s="4" t="inlineStr">
-        <is>
-          <t>Tinggi (telp/alamat), Sedang (email)</t>
-        </is>
-      </c>
-      <c r="N42" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O42" s="9" t="n"/>
-      <c r="P42" s="6" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="n">
+      <c r="L48" s="24" t="inlineStr">
+        <is>
+          <t>kibsons.com</t>
+        </is>
+      </c>
+      <c r="M48" s="20" t="inlineStr">
+        <is>
+          <t>Tinggi</t>
+        </is>
+      </c>
+      <c r="N48" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O48" s="26" t="n"/>
+      <c r="P48" s="23" t="n"/>
+    </row>
+    <row r="49" ht="34" customHeight="1">
+      <c r="A49" s="20" t="n">
         <v>39</v>
       </c>
-      <c r="B43" s="5" t="inlineStr">
+      <c r="B49" s="21" t="inlineStr">
         <is>
           <t>MPF Foodstuff Trading (Meridian PF)</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C49" s="20" t="inlineStr">
         <is>
           <t>UAE</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="D49" s="22" t="inlineStr">
         <is>
           <t>Dubai</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
+      <c r="E49" s="20" t="inlineStr">
         <is>
           <t>Distributor</t>
         </is>
       </c>
-      <c r="F43" s="4" t="inlineStr">
+      <c r="F49" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G43" s="5" t="inlineStr">
+      <c r="G49" s="22" t="inlineStr">
         <is>
           <t>Buah musiman &amp; eksotis</t>
         </is>
       </c>
-      <c r="H43" s="6" t="n"/>
-      <c r="I43" s="7" t="inlineStr">
+      <c r="H49" s="23" t="n"/>
+      <c r="I49" s="23" t="inlineStr">
         <is>
           <t>Purchase@meridianpf.com</t>
         </is>
       </c>
-      <c r="J43" s="7" t="inlineStr">
+      <c r="J49" s="23" t="inlineStr">
         <is>
           <t>+971 4 564 4106</t>
         </is>
       </c>
-      <c r="K43" s="5" t="inlineStr">
+      <c r="K49" s="22" t="inlineStr">
         <is>
           <t>Warehouse #21, Warsan 1, Dubai, PO Box 455012</t>
         </is>
       </c>
-      <c r="L43" s="8" t="inlineStr">
-        <is>
-          <t>https://meridianpf.com/contact-us/</t>
-        </is>
-      </c>
-      <c r="M43" s="4" t="inlineStr">
+      <c r="L49" s="24" t="inlineStr">
+        <is>
+          <t>meridianpf.com</t>
+        </is>
+      </c>
+      <c r="M49" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N43" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O43" s="9" t="n"/>
-      <c r="P43" s="6" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="n">
+      <c r="N49" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O49" s="26" t="n"/>
+      <c r="P49" s="23" t="n"/>
+    </row>
+    <row r="50" ht="34" customHeight="1">
+      <c r="A50" s="20" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="5" t="inlineStr">
+      <c r="B50" s="21" t="inlineStr">
         <is>
           <t>Shabab Al Aweer Foodstuff Trading L.L.C.</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C50" s="20" t="inlineStr">
         <is>
           <t>UAE</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="D50" s="22" t="inlineStr">
         <is>
           <t>Dubai (Al Aweer)</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
+      <c r="E50" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F44" s="4" t="inlineStr">
+      <c r="F50" s="20" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="G44" s="5" t="inlineStr">
+      <c r="G50" s="22" t="inlineStr">
         <is>
           <t>Impor/ekspor dan suplai buah &amp; sayur</t>
         </is>
       </c>
-      <c r="H44" s="6" t="n"/>
-      <c r="I44" s="7" t="n"/>
-      <c r="J44" s="7" t="n"/>
-      <c r="K44" s="5" t="inlineStr">
+      <c r="H50" s="23" t="n"/>
+      <c r="I50" s="23" t="n"/>
+      <c r="J50" s="23" t="n"/>
+      <c r="K50" s="22" t="inlineStr">
         <is>
           <t>Shop 23, Block 6, Fruits &amp; Vegetables Market, Al Aweer, Dubai</t>
         </is>
       </c>
-      <c r="L44" s="8" t="inlineStr">
-        <is>
-          <t>https://shababalaweer.ae/contact-us/</t>
-        </is>
-      </c>
-      <c r="M44" s="4" t="inlineStr">
+      <c r="L50" s="24" t="inlineStr">
+        <is>
+          <t>shababalaweer.ae</t>
+        </is>
+      </c>
+      <c r="M50" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N44" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O44" s="9" t="n"/>
-      <c r="P44" s="6" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="4" t="n">
+      <c r="N50" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O50" s="26" t="n"/>
+      <c r="P50" s="23" t="n"/>
+    </row>
+    <row r="51" ht="34" customHeight="1">
+      <c r="A51" s="20" t="n">
         <v>41</v>
       </c>
-      <c r="B45" s="5" t="inlineStr">
+      <c r="B51" s="21" t="inlineStr">
         <is>
           <t>Alghanim Sons Group – Fresh Produce</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C51" s="20" t="inlineStr">
         <is>
           <t>Kuwait</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="D51" s="22" t="inlineStr">
         <is>
           <t>Kuwait City</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
+      <c r="E51" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F45" s="4" t="inlineStr">
+      <c r="F51" s="20" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="G45" s="5" t="inlineStr">
+      <c r="G51" s="22" t="inlineStr">
         <is>
           <t>Divisi impor/distribusi produk segar</t>
         </is>
       </c>
-      <c r="H45" s="6" t="n"/>
-      <c r="I45" s="7" t="inlineStr">
+      <c r="H51" s="23" t="n"/>
+      <c r="I51" s="23" t="inlineStr">
         <is>
           <t>info@alghanimsons.com</t>
         </is>
       </c>
-      <c r="J45" s="7" t="inlineStr">
+      <c r="J51" s="23" t="inlineStr">
         <is>
           <t>+965 2228 2830</t>
         </is>
       </c>
-      <c r="K45" s="5" t="inlineStr">
+      <c r="K51" s="22" t="inlineStr">
         <is>
           <t>Safat 13097, Kuwait</t>
         </is>
       </c>
-      <c r="L45" s="8" t="inlineStr">
-        <is>
-          <t>https://www.alghanimsons.com/contact</t>
-        </is>
-      </c>
-      <c r="M45" s="4" t="inlineStr">
+      <c r="L51" s="24" t="inlineStr">
+        <is>
+          <t>alghanimsons.com</t>
+        </is>
+      </c>
+      <c r="M51" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N45" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O45" s="9" t="n"/>
-      <c r="P45" s="6" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="4" t="n">
+      <c r="N51" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O51" s="26" t="n"/>
+      <c r="P51" s="23" t="n"/>
+    </row>
+    <row r="52" ht="34" customHeight="1">
+      <c r="A52" s="20" t="n">
         <v>42</v>
       </c>
-      <c r="B46" s="5" t="inlineStr">
+      <c r="B52" s="21" t="inlineStr">
         <is>
           <t>Fresh Fruit Oman</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
+      <c r="C52" s="20" t="inlineStr">
         <is>
           <t>Oman</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D52" s="22" t="inlineStr">
         <is>
           <t>Muscat</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
+      <c r="E52" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F46" s="4" t="inlineStr">
+      <c r="F52" s="20" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="G46" s="5" t="inlineStr">
+      <c r="G52" s="22" t="inlineStr">
         <is>
           <t>Importir, grosir, manajemen ritel buah &amp; sayur</t>
         </is>
       </c>
-      <c r="H46" s="6" t="n"/>
-      <c r="I46" s="7" t="n"/>
-      <c r="J46" s="7" t="n"/>
-      <c r="K46" s="5" t="inlineStr">
+      <c r="H52" s="23" t="n"/>
+      <c r="I52" s="23" t="n"/>
+      <c r="J52" s="23" t="n"/>
+      <c r="K52" s="22" t="inlineStr">
         <is>
           <t>Mawaleh Central Market, Muscat, Oman (pasar pindah ke Khazaen 2024)</t>
         </is>
       </c>
-      <c r="L46" s="8" t="inlineStr">
-        <is>
-          <t>https://freshfruitoman.com/</t>
-        </is>
-      </c>
-      <c r="M46" s="4" t="inlineStr">
+      <c r="L52" s="24" t="inlineStr">
+        <is>
+          <t>freshfruitoman.com</t>
+        </is>
+      </c>
+      <c r="M52" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N46" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O46" s="9" t="n"/>
-      <c r="P46" s="6" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="4" t="n">
+      <c r="N52" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O52" s="26" t="n"/>
+      <c r="P52" s="23" t="n"/>
+    </row>
+    <row r="53" ht="30" customHeight="1">
+      <c r="A53" s="20" t="n">
         <v>43</v>
       </c>
-      <c r="B47" s="5" t="inlineStr">
+      <c r="B53" s="21" t="inlineStr">
         <is>
           <t>Redcolt Trading</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
+      <c r="C53" s="20" t="inlineStr">
         <is>
           <t>Qatar</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr">
+      <c r="D53" s="22" t="inlineStr">
         <is>
           <t>Doha</t>
         </is>
       </c>
-      <c r="E47" s="4" t="inlineStr">
+      <c r="E53" s="20" t="inlineStr">
         <is>
           <t>Importir</t>
         </is>
       </c>
-      <c r="F47" s="4" t="inlineStr">
+      <c r="F53" s="20" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="G47" s="5" t="inlineStr">
+      <c r="G53" s="22" t="inlineStr">
         <is>
           <t>Buah, sayur, produk makanan</t>
         </is>
       </c>
-      <c r="H47" s="6" t="n"/>
-      <c r="I47" s="7" t="n"/>
-      <c r="J47" s="7" t="n"/>
-      <c r="K47" s="5" t="n"/>
-      <c r="L47" s="8" t="inlineStr">
-        <is>
-          <t>https://redcoltqatar.com/</t>
-        </is>
-      </c>
-      <c r="M47" s="4" t="inlineStr">
-        <is>
-          <t>Tidak ditemukan</t>
-        </is>
-      </c>
-      <c r="N47" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O47" s="9" t="n"/>
-      <c r="P47" s="6" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="4" t="n">
+      <c r="H53" s="23" t="n"/>
+      <c r="I53" s="23" t="n"/>
+      <c r="J53" s="23" t="n"/>
+      <c r="K53" s="22" t="n"/>
+      <c r="L53" s="24" t="inlineStr">
+        <is>
+          <t>redcoltqatar.com</t>
+        </is>
+      </c>
+      <c r="M53" s="20" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N53" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O53" s="26" t="n"/>
+      <c r="P53" s="23" t="n"/>
+    </row>
+    <row r="54" ht="47" customHeight="1">
+      <c r="A54" s="20" t="n">
         <v>44</v>
       </c>
-      <c r="B48" s="5" t="inlineStr">
+      <c r="B54" s="21" t="inlineStr">
         <is>
           <t>Tamimi Markets</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C54" s="20" t="inlineStr">
         <is>
           <t>Saudi Arabia</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D54" s="22" t="inlineStr">
         <is>
           <t>Al Khobar</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
+      <c r="E54" s="20" t="inlineStr">
         <is>
           <t>Retail/Supermarket</t>
         </is>
       </c>
-      <c r="F48" s="4" t="inlineStr">
+      <c r="F54" s="20" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="G48" s="5" t="inlineStr">
+      <c r="G54" s="22" t="inlineStr">
         <is>
           <t>Supermarket premium, impor langsung</t>
         </is>
       </c>
-      <c r="H48" s="6" t="n"/>
-      <c r="I48" s="7" t="inlineStr">
+      <c r="H54" s="23" t="n"/>
+      <c r="I54" s="23" t="inlineStr">
         <is>
           <t>customerservice@tamimimarkets.com</t>
         </is>
       </c>
-      <c r="J48" s="7" t="inlineStr">
-        <is>
-          <t>+966 13 831 5100; CS 800 303 0010</t>
-        </is>
-      </c>
-      <c r="K48" s="5" t="inlineStr">
+      <c r="J54" s="23" t="inlineStr">
+        <is>
+          <t>+966 13 831 5100
+CS 800 303 0010</t>
+        </is>
+      </c>
+      <c r="K54" s="22" t="inlineStr">
         <is>
           <t>7107 King Fahd Bin Abdulaziz Rd, Al Rakah Al Janubiyah, Al Khobar 34227, Saudi Arabia</t>
         </is>
       </c>
-      <c r="L48" s="8" t="inlineStr">
-        <is>
-          <t>https://www.tamimimarkets.com/Contact</t>
-        </is>
-      </c>
-      <c r="M48" s="4" t="inlineStr">
-        <is>
-          <t>Tinggi (email), Sedang (telp/alamat)</t>
-        </is>
-      </c>
-      <c r="N48" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O48" s="9" t="n"/>
-      <c r="P48" s="6" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="4" t="n">
+      <c r="L54" s="24" t="inlineStr">
+        <is>
+          <t>tamimimarkets.com</t>
+        </is>
+      </c>
+      <c r="M54" s="20" t="inlineStr">
+        <is>
+          <t>Tinggi</t>
+        </is>
+      </c>
+      <c r="N54" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O54" s="26" t="n"/>
+      <c r="P54" s="23" t="n"/>
+    </row>
+    <row r="55" ht="34" customHeight="1">
+      <c r="A55" s="20" t="n">
         <v>45</v>
       </c>
-      <c r="B49" s="5" t="inlineStr">
+      <c r="B55" s="21" t="inlineStr">
         <is>
           <t>Al Maya Group (Al Maya Supermarkets)</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="C55" s="20" t="inlineStr">
         <is>
           <t>UAE</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr">
+      <c r="D55" s="22" t="inlineStr">
         <is>
           <t>Dubai</t>
         </is>
       </c>
-      <c r="E49" s="4" t="inlineStr">
+      <c r="E55" s="20" t="inlineStr">
         <is>
           <t>Retail/Supermarket</t>
         </is>
       </c>
-      <c r="F49" s="4" t="inlineStr">
+      <c r="F55" s="20" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="G49" s="5" t="inlineStr">
+      <c r="G55" s="22" t="inlineStr">
         <is>
           <t>Rantai supermarket (±40 gerai UAE)</t>
         </is>
       </c>
-      <c r="H49" s="6" t="n"/>
-      <c r="I49" s="7" t="inlineStr">
+      <c r="H55" s="23" t="n"/>
+      <c r="I55" s="23" t="inlineStr">
         <is>
           <t>info@almaya.ae</t>
         </is>
       </c>
-      <c r="J49" s="7" t="inlineStr">
+      <c r="J55" s="23" t="inlineStr">
         <is>
           <t>+971 4 823 0000</t>
         </is>
       </c>
-      <c r="K49" s="5" t="inlineStr">
+      <c r="K55" s="22" t="inlineStr">
         <is>
           <t>National Industries Park, Jebel Ali-3, Dubai, PO Box 8476, UAE</t>
         </is>
       </c>
-      <c r="L49" s="8" t="inlineStr">
-        <is>
-          <t>https://www.almaya.ae/contact-us.php</t>
-        </is>
-      </c>
-      <c r="M49" s="4" t="inlineStr">
+      <c r="L55" s="24" t="inlineStr">
+        <is>
+          <t>almaya.ae</t>
+        </is>
+      </c>
+      <c r="M55" s="20" t="inlineStr">
         <is>
           <t>Tinggi</t>
         </is>
       </c>
-      <c r="N49" s="6" t="inlineStr">
-        <is>
-          <t>Baru</t>
-        </is>
-      </c>
-      <c r="O49" s="9" t="n"/>
-      <c r="P49" s="6" t="n"/>
+      <c r="N55" s="25" t="inlineStr">
+        <is>
+          <t>Baru</t>
+        </is>
+      </c>
+      <c r="O55" s="26" t="n"/>
+      <c r="P55" s="23" t="n"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F5:F249">
+  <mergeCells count="21">
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="O7:P7"/>
+    <mergeCell ref="J5:K5"/>
+    <mergeCell ref="L5:N5"/>
+    <mergeCell ref="B8:P8"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="L4:N4"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="O5:P5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="C7:E7"/>
+    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="L7:N7"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="A2:P2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="F11:F255">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"A"</formula>
     </cfRule>
@@ -3566,87 +3872,97 @@
       <formula>"C"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M5:M249">
-    <cfRule type="expression" priority="4" dxfId="3">
-      <formula>LEFT(M5,6)="Tinggi"</formula>
+  <conditionalFormatting sqref="M11:M255">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+      <formula>"Tinggi"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" dxfId="4">
-      <formula>LEFT(M5,6)="Sedang"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="6" dxfId="5">
-      <formula>LEFT(M5,5)="Tidak"</formula>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="4">
+      <formula>"Sedang"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N5:N249">
-    <cfRule type="cellIs" priority="7" operator="equal" dxfId="3">
+  <conditionalFormatting sqref="N11:N255">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="0">
       <formula>"Deal"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O5:O249">
-    <cfRule type="expression" priority="8" dxfId="6">
-      <formula>AND(O5&lt;&gt;"",O5&lt;=TODAY(),N5&lt;&gt;"Deal",N5&lt;&gt;"Tidak Tertarik")</formula>
+  <conditionalFormatting sqref="O11:O255">
+    <cfRule type="expression" priority="7" dxfId="5">
+      <formula>AND(O11&lt;&gt;"",O11&lt;=TODAY(),N11&lt;&gt;"Deal",N11&lt;&gt;"Tidak Tertarik")</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="3">
-    <dataValidation sqref="N5:N249" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="4">
+    <dataValidation sqref="N11:N255" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Baru,Dihubungi,Negosiasi,Kirim Sampel,Deal,Tidak Tertarik"</formula1>
     </dataValidation>
-    <dataValidation sqref="F5:F249" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F11:F255" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"A,B,C"</formula1>
     </dataValidation>
-    <dataValidation sqref="E5:E249" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E11:E255" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Importir,Distributor,Wholesaler,Retail/Supermarket,E-commerce"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M11:M255" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Tinggi,Sedang,-"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L11" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L12" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L13" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L14" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L15" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L16" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L17" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L18" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L19" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L20" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L21" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L22" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L23" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L24" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L25" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L26" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L27" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L28" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L29" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L30" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L31" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L32" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L33" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L34" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L35" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L36" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L37" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L38" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L39" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L40" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L41" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L42" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L43" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L50" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L51" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L52" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L53" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L54" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L55" r:id="rId45"/>
   </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 Halaman &amp;P dari &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId46"/>
   </tableParts>

</xml_diff>